<commit_message>
backup before Work test
</commit_message>
<xml_diff>
--- a/Data/stocks-in-port.xlsx
+++ b/Data/stocks-in-port.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c8862359375ebd62/A4/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="11_E26E99DC1DCDF12C2843E0BFFB6C5B8E956E9E70" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E434B730-6777-42BF-9686-2A2778F083B3}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="11_E26E99DC1DCDF12C2843E0BFFB6C5B8E956E9E70" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AC22D41-E96B-4350-9D44-27A8418A76A1}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12552" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="2172" windowWidth="4560" windowHeight="9564" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -303,7 +303,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -340,12 +340,6 @@
     <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -361,10 +355,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -897,7 +887,7 @@
         <v>3</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="X3" s="5">
         <v>2</v>
@@ -1057,7 +1047,7 @@
         <v>2</v>
       </c>
       <c r="W5" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="X5">
         <v>2</v>
@@ -1552,82 +1542,82 @@
       </c>
     </row>
     <row r="12" spans="1:29">
-      <c r="A12" s="24" t="s">
+      <c r="A12" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="24">
+      <c r="B12">
         <v>2026</v>
       </c>
-      <c r="C12" s="24">
-        <v>2</v>
-      </c>
-      <c r="D12" s="25">
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12" s="2">
         <v>233958</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="2">
         <v>246468</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="2">
         <v>-12510</v>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="2">
         <v>486159</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="2">
         <v>576497</v>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="2">
         <v>-90338</v>
       </c>
-      <c r="J12" s="26">
+      <c r="J12" s="7">
         <v>44952</v>
       </c>
-      <c r="K12" s="27">
+      <c r="K12" s="17">
         <v>7000</v>
       </c>
-      <c r="L12" s="24">
+      <c r="L12">
         <v>37.700000000000003</v>
       </c>
-      <c r="M12" s="24">
+      <c r="M12">
         <v>11.4</v>
       </c>
-      <c r="N12" s="25">
+      <c r="N12" s="2">
         <v>263900</v>
       </c>
-      <c r="O12" s="25">
+      <c r="O12" s="2">
         <v>79800</v>
       </c>
-      <c r="P12" s="25">
+      <c r="P12" s="2">
         <v>-184100</v>
       </c>
-      <c r="Q12" s="24">
+      <c r="Q12">
         <v>0.7</v>
       </c>
-      <c r="R12" s="28">
+      <c r="R12" s="3">
         <v>6.1403508771929802</v>
       </c>
-      <c r="S12" s="24">
+      <c r="S12">
         <v>-5.08</v>
       </c>
-      <c r="T12" s="24">
+      <c r="T12">
         <v>-15.67</v>
       </c>
-      <c r="U12" s="29">
+      <c r="U12" s="1">
         <v>-69.761273209549103</v>
       </c>
-      <c r="V12" s="24">
+      <c r="V12">
         <v>4</v>
       </c>
-      <c r="W12" s="24" t="s">
+      <c r="W12" t="s">
         <v>28</v>
       </c>
-      <c r="X12" s="24">
+      <c r="X12">
         <v>1</v>
       </c>
-      <c r="Y12" s="24" t="s">
+      <c r="Y12" t="s">
         <v>27</v>
       </c>
-      <c r="Z12" s="24">
+      <c r="Z12">
         <v>245</v>
       </c>
     </row>

</xml_diff>